<commit_message>
fix: sincronizar arquivos raiz de franquias e lojas-proprias para corrigir deploy vercel
</commit_message>
<xml_diff>
--- a/lojas-proprias/pwr_reports/Keys Summary - Lojas Corporativas (Stores)(2026-07-27 - 2026-07-31).xlsx
+++ b/lojas-proprias/pwr_reports/Keys Summary - Lojas Corporativas (Stores)(2026-07-27 - 2026-07-31).xlsx
@@ -146,10 +146,10 @@
     <t>International Not Used</t>
   </si>
   <si>
-    <t>RJ</t>
-  </si>
-  <si>
-    <t>Rio de Janeiro</t>
+    <t>GO</t>
+  </si>
+  <si>
+    <t>Brasilia</t>
   </si>
   <si>
     <t>Soares,Fernando</t>
@@ -179,97 +179,190 @@
     <t>I</t>
   </si>
   <si>
+    <t>Ramos,Bernardo Guimaraes Batista</t>
+  </si>
+  <si>
     <t>Pulse Other</t>
   </si>
   <si>
-    <t>Lautersztajn,Andres</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>Belo Horizonte</t>
-  </si>
-  <si>
-    <t>Neto,Orestes Miraglia</t>
-  </si>
-  <si>
-    <t>Rio De Janeiro</t>
-  </si>
-  <si>
-    <t>Silva,Jairo and Carmem</t>
-  </si>
-  <si>
-    <t>RIO DE JANEIRO</t>
-  </si>
-  <si>
-    <t>22
-21</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>R$ 751.600,40</t>
-  </si>
-  <si>
-    <t>R$ 34.163,65
-R$ 34.601,97</t>
-  </si>
-  <si>
-    <t>7.0%
-8.3%</t>
-  </si>
-  <si>
-    <t>364.0</t>
-  </si>
-  <si>
-    <t>8.4%</t>
-  </si>
-  <si>
-    <t>32.8%</t>
-  </si>
-  <si>
-    <t>(0.1%)</t>
-  </si>
-  <si>
-    <t>3.2%</t>
-  </si>
-  <si>
-    <t>0.2%</t>
-  </si>
-  <si>
-    <t>26.6</t>
-  </si>
-  <si>
-    <t>75.1%</t>
-  </si>
-  <si>
-    <t>8.1%</t>
-  </si>
-  <si>
-    <t>7.8</t>
-  </si>
-  <si>
-    <t>4.4</t>
-  </si>
-  <si>
-    <t>12.0</t>
-  </si>
-  <si>
-    <t>19.1</t>
-  </si>
-  <si>
-    <t>78.5%</t>
-  </si>
-  <si>
-    <t>-R$ 20.151,98</t>
-  </si>
-  <si>
-    <t>4.68</t>
-  </si>
-  <si>
-    <t>3.71</t>
+    <t>GUARA II</t>
+  </si>
+  <si>
+    <t>Silva de Carvalho,Flavio Roberto and Rodrigo Jose</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>São Luis</t>
+  </si>
+  <si>
+    <t>Lazera,Áurea</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>Campo Grande</t>
+  </si>
+  <si>
+    <t>Hermeto,Adriano</t>
+  </si>
+  <si>
+    <t>Cohama - Sao Luis</t>
+  </si>
+  <si>
+    <t>PEREIRA,MARCIA MARIA</t>
+  </si>
+  <si>
+    <t>BARROSO V BOAS DE CARVALHO,ANDREA LOPES</t>
+  </si>
+  <si>
+    <t>Goiania</t>
+  </si>
+  <si>
+    <t>Cortez,Matheus</t>
+  </si>
+  <si>
+    <t>Lessa,Lincoln</t>
+  </si>
+  <si>
+    <t>Matheus Cortes,Luis</t>
+  </si>
+  <si>
+    <t>Cuiaba</t>
+  </si>
+  <si>
+    <t>Nespolo,Cinara and Jorge Carvalho</t>
+  </si>
+  <si>
+    <t>Porto Velho</t>
+  </si>
+  <si>
+    <t>Rezende,Daniel</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>Rio Branco</t>
+  </si>
+  <si>
+    <t>Pacific,Nogroup</t>
+  </si>
+  <si>
+    <t>BARCELOS,JUMARA DA COSTA NOLASCO</t>
+  </si>
+  <si>
+    <t>Boa Vista</t>
+  </si>
+  <si>
+    <t>Veiga,Mauricio</t>
+  </si>
+  <si>
+    <t>Cuiabá</t>
+  </si>
+  <si>
+    <t>RO</t>
+  </si>
+  <si>
+    <t>SOLIGO,MATHEUS PINHEIRO</t>
+  </si>
+  <si>
+    <t>BRASILIA</t>
+  </si>
+  <si>
+    <t>Risuenho,Igor and Vinicius Costa</t>
+  </si>
+  <si>
+    <t>TAGUATINGA</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>PARAUAPEBAS</t>
+  </si>
+  <si>
+    <t>Duarte,Patricia</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>TANGARA DA SERRA</t>
+  </si>
+  <si>
+    <t>Dos Santos,Josemar Carmerino andMarcioandElisandro</t>
+  </si>
+  <si>
+    <t>25
+23</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>R$ 653.250,14</t>
+  </si>
+  <si>
+    <t>R$ 26.130,01
+R$ 26.668,47</t>
+  </si>
+  <si>
+    <t>(5.9%)
+(4.0%)</t>
+  </si>
+  <si>
+    <t>263.2</t>
+  </si>
+  <si>
+    <t>(10.3%)</t>
+  </si>
+  <si>
+    <t>486.3%</t>
+  </si>
+  <si>
+    <t>452.5%</t>
+  </si>
+  <si>
+    <t>2.5%</t>
+  </si>
+  <si>
+    <t>0.0%</t>
+  </si>
+  <si>
+    <t>26.2</t>
+  </si>
+  <si>
+    <t>76.1%</t>
+  </si>
+  <si>
+    <t>9.0%</t>
+  </si>
+  <si>
+    <t>5.5</t>
+  </si>
+  <si>
+    <t>6.3</t>
+  </si>
+  <si>
+    <t>11.6</t>
+  </si>
+  <si>
+    <t>18.4</t>
+  </si>
+  <si>
+    <t>75.0%</t>
+  </si>
+  <si>
+    <t>-R$ 10.644,06</t>
+  </si>
+  <si>
+    <t>2.96</t>
+  </si>
+  <si>
+    <t>3.00</t>
   </si>
   <si>
     <t>1</t>
@@ -687,7 +780,7 @@
     <col min="2" max="2" width="2.86" customWidth="1"/>
     <col min="3" max="3" width="17.86" customWidth="1"/>
     <col min="4" max="4" width="4.43" customWidth="1"/>
-    <col min="5" max="5" width="15.14" customWidth="1"/>
+    <col min="5" max="5" width="19.43" customWidth="1"/>
     <col min="6" max="6" width="13.29" customWidth="1"/>
     <col min="7" max="7" width="5.57" customWidth="1"/>
     <col min="8" max="8" width="12.71" customWidth="1"/>
@@ -726,7 +819,7 @@
     <col min="41" max="41" width="9.43" customWidth="1"/>
     <col min="42" max="42" width="14.57" customWidth="1"/>
     <col min="43" max="43" width="7.14" customWidth="1"/>
-    <col min="44" max="44" width="18.71" customWidth="1"/>
+    <col min="44" max="44" width="42.43" customWidth="1"/>
     <col min="45" max="45" width="11.14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -869,7 +962,7 @@
     </row>
     <row r="2" ht="13.5" customHeight="1">
       <c r="A2" s="2">
-        <v>19504</v>
+        <v>19550</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
@@ -909,68 +1002,64 @@
         <v>52</v>
       </c>
       <c r="O2" s="5">
-        <v>42129.239999999998</v>
+        <v>21834.939999999999</v>
       </c>
       <c r="P2" s="5">
-        <v>42129.239999999998</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>-0.042058113764074756</v>
-      </c>
+        <v>21834.939999999999</v>
+      </c>
+      <c r="Q2" s="6"/>
       <c r="R2" s="7">
-        <v>422</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0.021791767554479424</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="S2" s="6"/>
       <c r="T2" s="6">
-        <v>0.3427340298566981</v>
+        <v>0.37830422249843604</v>
       </c>
       <c r="U2" s="6">
-        <v>0.010092852375214935</v>
+        <v>-0.036660050359652925</v>
       </c>
       <c r="V2" s="6">
-        <v>0.01557275896740601</v>
+        <v>0.024433064620282906</v>
       </c>
       <c r="W2" s="6">
-        <v>-0.010413705540380031</v>
+        <v>-0.012805416456376799</v>
       </c>
       <c r="X2" s="8">
-        <v>20.152573333333333</v>
+        <v>22.145096470588236</v>
       </c>
       <c r="Y2" s="6">
-        <v>0.92280701754385963</v>
+        <v>0.90588235294117647</v>
       </c>
       <c r="Z2" s="6">
-        <v>0</v>
+        <v>0.023529411764705882</v>
       </c>
       <c r="AA2" s="8">
-        <v>4.8671851674641147</v>
+        <v>2.4474420792079208</v>
       </c>
       <c r="AB2" s="8">
-        <v>3.1573287234042553</v>
+        <v>4.6795168674698795</v>
       </c>
       <c r="AC2" s="8">
-        <v>8.6383220000000005</v>
+        <v>7.7614530000000004</v>
       </c>
       <c r="AD2" s="8">
-        <v>15.132222105263157</v>
+        <v>13.890784705882352</v>
       </c>
       <c r="AE2" s="6">
-        <v>0.93684210526315792</v>
+        <v>0.85882352941176465</v>
       </c>
       <c r="AF2" s="9"/>
       <c r="AG2" s="5">
-        <v>-743.10000000000002</v>
+        <v>-89.799999999999997</v>
       </c>
       <c r="AH2" s="10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AI2" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AJ2" s="12">
-        <v>46035</v>
+        <v>46099</v>
       </c>
       <c t="s" r="AK2" s="4">
         <v>52</v>
@@ -993,14 +1082,16 @@
       <c t="s" r="AQ2" s="4">
         <v>55</v>
       </c>
-      <c r="AR2" s="4"/>
+      <c t="s" r="AR2" s="4">
+        <v>56</v>
+      </c>
       <c t="s" r="AS2" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" ht="13.5" customHeight="1">
       <c r="A3" s="2">
-        <v>19505</v>
+        <v>19551</v>
       </c>
       <c r="B3" s="3">
         <v>0</v>
@@ -1040,68 +1131,66 @@
         <v>52</v>
       </c>
       <c r="O3" s="5">
-        <v>30934.07</v>
+        <v>38000.760000000002</v>
       </c>
       <c r="P3" s="5">
-        <v>30934.07</v>
+        <v>38000.760000000002</v>
       </c>
       <c r="Q3" s="6">
-        <v>0.026157775298692787</v>
+        <v>-0.11935103958530602</v>
       </c>
       <c r="R3" s="7">
         <v>347</v>
       </c>
       <c r="S3" s="6">
-        <v>-0.0085714285714285632</v>
+        <v>-0.13466334164588534</v>
       </c>
       <c r="T3" s="6">
-        <v>0.38970023666462256</v>
+        <v>-0.40034751410234953</v>
       </c>
       <c r="U3" s="6">
-        <v>0.008359210411045169</v>
+        <v>-0.74340644239746778</v>
       </c>
       <c r="V3" s="6">
-        <v>0.036029927520045052</v>
+        <v>0.020284607465745421</v>
       </c>
       <c r="W3" s="6">
-        <v>-0.010991366477156093</v>
+        <v>0.0090579898928337226</v>
       </c>
       <c r="X3" s="8">
-        <v>23.458811877394634</v>
+        <v>22.257657657657656</v>
       </c>
       <c r="Y3" s="6">
-        <v>0.80842911877394641</v>
+        <v>0.89639639639639634</v>
       </c>
       <c r="Z3" s="6">
-        <v>0.011494252873563218</v>
+        <v>0.022522522522522521</v>
       </c>
       <c r="AA3" s="8">
-        <v>7.0997575581395349</v>
+        <v>3.019857142857143</v>
       </c>
       <c r="AB3" s="8">
-        <v>3.9356407692307696</v>
+        <v>5.360982949308756</v>
       </c>
       <c r="AC3" s="8">
-        <v>11.419763</v>
+        <v>8.3621180000000006</v>
       </c>
       <c r="AD3" s="8">
-        <v>16.353320689655174</v>
+        <v>16.151726576576579</v>
       </c>
       <c r="AE3" s="6">
-        <v>0.87739463601532564</v>
+        <v>0.90090090090090091</v>
       </c>
       <c r="AF3" s="9"/>
       <c r="AG3" s="5">
-        <v>-292.10000000000002</v>
+        <v>0</v>
       </c>
       <c r="AH3" s="10">
         <v>5</v>
       </c>
-      <c r="AI3" s="11">
-        <v>4</v>
-      </c>
+      <c r="AI3" s="11"/>
       <c r="AJ3" s="12">
-        <v>46154</v>
+        <v>46010</v>
       </c>
       <c t="s" r="AK3" s="4">
         <v>52</v>
@@ -1124,17 +1213,19 @@
       <c t="s" r="AQ3" s="4">
         <v>55</v>
       </c>
-      <c r="AR3" s="4"/>
+      <c t="s" r="AR3" s="4">
+        <v>56</v>
+      </c>
       <c t="s" r="AS3" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="2">
-        <v>19507</v>
+        <v>19552</v>
       </c>
       <c r="B4" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c t="s" r="C4" s="4">
         <v>44</v>
@@ -1171,68 +1262,66 @@
         <v>52</v>
       </c>
       <c r="O4" s="5">
-        <v>15609.41</v>
+        <v>58369.679999999993</v>
       </c>
       <c r="P4" s="5">
-        <v>15609.41</v>
+        <v>58369.679999999993</v>
       </c>
       <c r="Q4" s="6">
-        <v>-0.024042841199328535</v>
+        <v>0.041725465196237765</v>
       </c>
       <c r="R4" s="7">
-        <v>160</v>
+        <v>574</v>
       </c>
       <c r="S4" s="6">
-        <v>0.019108280254777066</v>
+        <v>0.012345679012345734</v>
       </c>
       <c r="T4" s="6">
-        <v>0.37223505564912446</v>
+        <v>0.28168302104791393</v>
       </c>
       <c r="U4" s="6">
-        <v>0.0031147621851178231</v>
+        <v>-0.045129461048955551</v>
       </c>
       <c r="V4" s="6">
-        <v>0.021751462739462924</v>
+        <v>0.022425118657494778</v>
       </c>
       <c r="W4" s="6">
-        <v>-0.010068445892573774</v>
+        <v>0.0080584132035673318</v>
       </c>
       <c r="X4" s="8">
-        <v>23.530059821428573</v>
+        <v>23.090835036496347</v>
       </c>
       <c r="Y4" s="6">
-        <v>0.9107142857142857</v>
+        <v>0.88807785888077861</v>
       </c>
       <c r="Z4" s="6">
-        <v>0.0089285714285714281</v>
+        <v>0.0097323600973236012</v>
       </c>
       <c r="AA4" s="8">
-        <v>6.7771764331210189</v>
+        <v>2.4572439929328622</v>
       </c>
       <c r="AB4" s="8">
-        <v>2.8245535714285714</v>
+        <v>5.3131300000000001</v>
       </c>
       <c r="AC4" s="8">
-        <v>9.8476180000000006</v>
+        <v>7.3831340000000001</v>
       </c>
       <c r="AD4" s="8">
-        <v>16.800149107142857</v>
+        <v>13.741605839416058</v>
       </c>
       <c r="AE4" s="6">
-        <v>0.9196428571428571</v>
+        <v>0.88321167883211682</v>
       </c>
       <c r="AF4" s="9"/>
       <c r="AG4" s="5">
-        <v>-71.5</v>
+        <v>0</v>
       </c>
       <c r="AH4" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI4" s="11">
-        <v>3</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="AI4" s="11"/>
       <c r="AJ4" s="12">
-        <v>45985</v>
+        <v>46013</v>
       </c>
       <c t="s" r="AK4" s="4">
         <v>52</v>
@@ -1255,14 +1344,16 @@
       <c t="s" r="AQ4" s="4">
         <v>55</v>
       </c>
-      <c r="AR4" s="4"/>
+      <c t="s" r="AR4" s="4">
+        <v>56</v>
+      </c>
       <c t="s" r="AS4" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="2">
-        <v>19508</v>
+        <v>19553</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
@@ -1270,11 +1361,9 @@
       <c t="s" r="C5" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D5" s="4">
-        <v>45</v>
-      </c>
+      <c r="D5" s="4"/>
       <c t="s" r="E5" s="4">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c t="s" r="F5" s="4">
         <v>47</v>
@@ -1302,68 +1391,66 @@
         <v>52</v>
       </c>
       <c r="O5" s="5">
-        <v>44731.550000000003</v>
+        <v>31314.359999999997</v>
       </c>
       <c r="P5" s="5">
-        <v>44731.550000000003</v>
+        <v>31314.359999999997</v>
       </c>
       <c r="Q5" s="6">
-        <v>0.037768547817014886</v>
+        <v>0.026851830597957038</v>
       </c>
       <c r="R5" s="7">
-        <v>469</v>
+        <v>279</v>
       </c>
       <c r="S5" s="6">
-        <v>0.015151515151515138</v>
+        <v>-0.076158940397350938</v>
       </c>
       <c r="T5" s="6">
-        <v>0.3458352102710503</v>
+        <v>0.33282896409187346</v>
       </c>
       <c r="U5" s="6">
-        <v>-0.0024163034815471406</v>
+        <v>-0.012686639611986322</v>
       </c>
       <c r="V5" s="6">
-        <v>0.02902535235197528</v>
+        <v>0.03499193341329665</v>
       </c>
       <c r="W5" s="6">
-        <v>-0.00021888353969401909</v>
+        <v>0.0030982590734730006</v>
       </c>
       <c r="X5" s="8">
-        <v>26.963161373390555</v>
+        <v>20.50708735632184</v>
       </c>
       <c r="Y5" s="6">
-        <v>0.79399141630901282</v>
+        <v>0.94252873563218387</v>
       </c>
       <c r="Z5" s="6">
-        <v>0.047210300429184553</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="8">
-        <v>7.0563953488372091</v>
+        <v>1.8490546099290781</v>
       </c>
       <c r="AB5" s="8">
-        <v>3.9949626666666664</v>
+        <v>3.2192682080924855</v>
       </c>
       <c r="AC5" s="8">
-        <v>12.528233999999999</v>
+        <v>5.5353750000000002</v>
       </c>
       <c r="AD5" s="8">
-        <v>18.752360515021461</v>
+        <v>11.918294827586207</v>
       </c>
       <c r="AE5" s="6">
-        <v>0.70386266094420602</v>
+        <v>0.97701149425287359</v>
       </c>
       <c r="AF5" s="9"/>
       <c r="AG5" s="5">
-        <v>-420.30000000000001</v>
+        <v>-157.80000000000001</v>
       </c>
       <c r="AH5" s="10">
         <v>5</v>
       </c>
-      <c r="AI5" s="11">
-        <v>2</v>
-      </c>
+      <c r="AI5" s="11"/>
       <c r="AJ5" s="12">
-        <v>46083</v>
+        <v>46154</v>
       </c>
       <c t="s" r="AK5" s="4">
         <v>52</v>
@@ -1387,15 +1474,15 @@
         <v>55</v>
       </c>
       <c t="s" r="AR5" s="4">
+        <v>59</v>
+      </c>
+      <c t="s" r="AS5" s="4">
         <v>57</v>
-      </c>
-      <c t="s" r="AS5" s="4">
-        <v>56</v>
       </c>
     </row>
     <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="2">
-        <v>19509</v>
+        <v>19595</v>
       </c>
       <c r="B6" s="3">
         <v>0</v>
@@ -1404,10 +1491,10 @@
         <v>44</v>
       </c>
       <c t="s" r="D6" s="4">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c t="s" r="E6" s="4">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c t="s" r="F6" s="4">
         <v>47</v>
@@ -1435,68 +1522,66 @@
         <v>52</v>
       </c>
       <c r="O6" s="5">
-        <v>38766.510000000002</v>
+        <v>60721.229999999996</v>
       </c>
       <c r="P6" s="5">
-        <v>38766.510000000002</v>
+        <v>60721.229999999996</v>
       </c>
       <c r="Q6" s="6">
-        <v>0.24620943989785116</v>
+        <v>-0.010195174407999663</v>
       </c>
       <c r="R6" s="7">
-        <v>425</v>
+        <v>588</v>
       </c>
       <c r="S6" s="6">
-        <v>0.17728531855955687</v>
+        <v>-0.054662379421221874</v>
       </c>
       <c r="T6" s="6">
-        <v>0.36324532953830507</v>
+        <v>0.3070468318905924</v>
       </c>
       <c r="U6" s="6">
-        <v>0.016921917913167835</v>
+        <v>-0.013457709931106466</v>
       </c>
       <c r="V6" s="6">
-        <v>0.022045407234233878</v>
+        <v>0.011464713412425935</v>
       </c>
       <c r="W6" s="6">
-        <v>0.0016463566103835502</v>
+        <v>-0.0027767635800526437</v>
       </c>
       <c r="X6" s="8">
-        <v>28.342497250859104</v>
+        <v>24.383520786516854</v>
       </c>
       <c r="Y6" s="6">
-        <v>0.71134020618556704</v>
+        <v>0.7247191011235955</v>
       </c>
       <c r="Z6" s="6">
-        <v>0.15463917525773196</v>
+        <v>0.061797752808988762</v>
       </c>
       <c r="AA6" s="8">
-        <v>9.5582344418052259</v>
+        <v>7.7298352733686073</v>
       </c>
       <c r="AB6" s="8">
-        <v>2.4525199312714778</v>
+        <v>4.2939482142857139</v>
       </c>
       <c r="AC6" s="8">
-        <v>13.525197</v>
+        <v>13.116580000000001</v>
       </c>
       <c r="AD6" s="8">
-        <v>20.752118900343643</v>
+        <v>19.487640449438203</v>
       </c>
       <c r="AE6" s="6">
-        <v>0.68041237113402064</v>
+        <v>0.8314606741573034</v>
       </c>
       <c r="AF6" s="9"/>
       <c r="AG6" s="5">
-        <v>-525.28999999999996</v>
+        <v>-694</v>
       </c>
       <c r="AH6" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI6" s="11">
-        <v>2</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="AI6" s="11"/>
       <c r="AJ6" s="12">
-        <v>45944</v>
+        <v>46000</v>
       </c>
       <c t="s" r="AK6" s="4">
         <v>52</v>
@@ -1519,26 +1604,28 @@
       <c t="s" r="AQ6" s="4">
         <v>55</v>
       </c>
-      <c r="AR6" s="4"/>
+      <c t="s" r="AR6" s="4">
+        <v>62</v>
+      </c>
       <c t="s" r="AS6" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="2">
-        <v>19511</v>
+        <v>19602</v>
       </c>
       <c r="B7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="s" r="C7" s="4">
         <v>44</v>
       </c>
       <c t="s" r="D7" s="4">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c t="s" r="E7" s="4">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c t="s" r="F7" s="4">
         <v>47</v>
@@ -1566,66 +1653,66 @@
         <v>52</v>
       </c>
       <c r="O7" s="5">
-        <v>41039.75</v>
+        <v>2174.0999999999999</v>
       </c>
       <c r="P7" s="5">
-        <v>41039.75</v>
+        <v>2174.0999999999999</v>
       </c>
       <c r="Q7" s="6">
-        <v>-0.013093899733673253</v>
+        <v>-0.52097140943382914</v>
       </c>
       <c r="R7" s="7">
-        <v>395</v>
+        <v>22</v>
       </c>
       <c r="S7" s="6">
-        <v>-0.031862745098039214</v>
+        <v>-0.53191489361702127</v>
       </c>
       <c r="T7" s="6">
-        <v>0.32130077303102478</v>
+        <v>0</v>
       </c>
       <c r="U7" s="6">
-        <v>0.0088205556807729093</v>
+        <v>-0.4283059656869509</v>
       </c>
       <c r="V7" s="6">
-        <v>0.031095230843267808</v>
+        <v>0.057641092866013523</v>
       </c>
       <c r="W7" s="6">
-        <v>-0.00040569204247101892</v>
+        <v>-0.17787705257347869</v>
       </c>
       <c r="X7" s="8">
-        <v>22.644852123552123</v>
+        <v>31.091674999999999</v>
       </c>
       <c r="Y7" s="6">
-        <v>0.60617760617760619</v>
+        <v>1</v>
       </c>
       <c r="Z7" s="6">
-        <v>0.0077220077220077222</v>
+        <v>0.25</v>
       </c>
       <c r="AA7" s="8">
-        <v>5.532861082474227</v>
+        <v>9.9801230769230767</v>
       </c>
       <c r="AB7" s="8">
-        <v>4.9688231372549021</v>
+        <v>9.7958374999999993</v>
       </c>
       <c r="AC7" s="8">
-        <v>10.891223</v>
+        <v>23.334720999999998</v>
       </c>
       <c r="AD7" s="8">
-        <v>16.922329343629347</v>
+        <v>25.4375</v>
       </c>
       <c r="AE7" s="6">
-        <v>0.86872586872586877</v>
+        <v>0.5</v>
       </c>
       <c r="AF7" s="9"/>
       <c r="AG7" s="5">
-        <v>-12036.540000000001</v>
+        <v>0</v>
       </c>
       <c r="AH7" s="10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AI7" s="11"/>
       <c r="AJ7" s="12">
-        <v>46078</v>
+        <v>46027</v>
       </c>
       <c t="s" r="AK7" s="4">
         <v>52</v>
@@ -1648,14 +1735,16 @@
       <c t="s" r="AQ7" s="4">
         <v>55</v>
       </c>
-      <c r="AR7" s="4"/>
+      <c t="s" r="AR7" s="4">
+        <v>65</v>
+      </c>
       <c t="s" r="AS7" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1">
       <c r="A8" s="2">
-        <v>19512</v>
+        <v>19617</v>
       </c>
       <c r="B8" s="3">
         <v>0</v>
@@ -1664,10 +1753,10 @@
         <v>44</v>
       </c>
       <c t="s" r="D8" s="4">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c t="s" r="E8" s="4">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c t="s" r="F8" s="4">
         <v>47</v>
@@ -1695,68 +1784,66 @@
         <v>52</v>
       </c>
       <c r="O8" s="5">
-        <v>37541.909999999996</v>
+        <v>52118.599999999999</v>
       </c>
       <c r="P8" s="5">
-        <v>37541.909999999996</v>
+        <v>52118.599999999999</v>
       </c>
       <c r="Q8" s="6">
-        <v>0.14104189392375943</v>
+        <v>0.16623789341167527</v>
       </c>
       <c r="R8" s="7">
-        <v>345</v>
+        <v>553</v>
       </c>
       <c r="S8" s="6">
-        <v>0.061538461538461542</v>
+        <v>0.077972709551656916</v>
       </c>
       <c r="T8" s="6">
-        <v>0.33240660371302361</v>
+        <v>0.34939915308546277</v>
       </c>
       <c r="U8" s="6">
-        <v>0.0004293548197201474</v>
+        <v>-0.015255883696031744</v>
       </c>
       <c r="V8" s="6">
-        <v>0.020443352509235676</v>
+        <v>0.02094125705602223</v>
       </c>
       <c r="W8" s="6">
-        <v>-0.0077989505595213457</v>
+        <v>0.0066214173059138196</v>
       </c>
       <c r="X8" s="8">
-        <v>23.011781465517242</v>
+        <v>34.601509448818902</v>
       </c>
       <c r="Y8" s="6">
-        <v>0.7931034482758621</v>
+        <v>0.75984251968503935</v>
       </c>
       <c r="Z8" s="6">
-        <v>0.012931034482758621</v>
+        <v>0.31496062992125984</v>
       </c>
       <c r="AA8" s="8">
-        <v>5.7787120943952806</v>
+        <v>10.553533583489681</v>
       </c>
       <c r="AB8" s="8">
-        <v>2.6148627705627709</v>
+        <v>8.0303274590163927</v>
       </c>
       <c r="AC8" s="8">
-        <v>8.9193499999999997</v>
+        <v>20.776292000000002</v>
       </c>
       <c r="AD8" s="8">
-        <v>15.840589224137931</v>
+        <v>26.119094488188978</v>
       </c>
       <c r="AE8" s="6">
-        <v>0.91379310344827591</v>
+        <v>0.46456692913385828</v>
       </c>
       <c r="AF8" s="9"/>
       <c r="AG8" s="5">
-        <v>-403.89999999999998</v>
+        <v>-1143</v>
       </c>
       <c r="AH8" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI8" s="11">
-        <v>4</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI8" s="11"/>
       <c r="AJ8" s="12">
-        <v>44774</v>
+        <v>46013</v>
       </c>
       <c t="s" r="AK8" s="4">
         <v>52</v>
@@ -1779,24 +1866,24 @@
       <c t="s" r="AQ8" s="4">
         <v>55</v>
       </c>
-      <c r="AR8" s="4"/>
+      <c t="s" r="AR8" s="4">
+        <v>62</v>
+      </c>
       <c t="s" r="AS8" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="2">
-        <v>19515</v>
+        <v>19647</v>
       </c>
       <c r="B9" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="s" r="C9" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D9" s="4">
-        <v>45</v>
-      </c>
+      <c r="D9" s="4"/>
       <c t="s" r="E9" s="4">
         <v>46</v>
       </c>
@@ -1826,68 +1913,66 @@
         <v>52</v>
       </c>
       <c r="O9" s="5">
-        <v>22662.579999999998</v>
+        <v>21882.260000000002</v>
       </c>
       <c r="P9" s="5">
-        <v>22662.579999999998</v>
+        <v>21882.260000000002</v>
       </c>
       <c r="Q9" s="6">
-        <v>-0.042230461464730529</v>
+        <v>0.04985932954118022</v>
       </c>
       <c r="R9" s="7">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="S9" s="6">
-        <v>-0.077551020408163307</v>
+        <v>-0.056680161943319818</v>
       </c>
       <c r="T9" s="6">
-        <v>0.32129076212858376</v>
+        <v>0</v>
       </c>
       <c r="U9" s="6">
-        <v>-0.019810736465133271</v>
+        <v>-0.37097356488772187</v>
       </c>
       <c r="V9" s="6">
-        <v>0.029664989599595456</v>
+        <v>0.026715613469541079</v>
       </c>
       <c r="W9" s="6">
-        <v>0.027010834600473557</v>
+        <v>-0.015711448451850952</v>
       </c>
       <c r="X9" s="8">
-        <v>56.651421022727277</v>
+        <v>27.454545454545453</v>
       </c>
       <c r="Y9" s="6">
-        <v>0.45454545454545453</v>
+        <v>0.76969696969696966</v>
       </c>
       <c r="Z9" s="6">
-        <v>0.42045454545454547</v>
+        <v>0.12121212121212122</v>
       </c>
       <c r="AA9" s="8">
-        <v>14.197835497835497</v>
+        <v>4.4450067510548523</v>
       </c>
       <c r="AB9" s="8">
-        <v>20.714583522727274</v>
+        <v>6.7118283870967739</v>
       </c>
       <c r="AC9" s="8">
-        <v>37.022540999999997</v>
+        <v>12.641301</v>
       </c>
       <c r="AD9" s="8">
-        <v>39.115000000000002</v>
+        <v>18.405151515151516</v>
       </c>
       <c r="AE9" s="6">
-        <v>0.32954545454545453</v>
+        <v>0.67272727272727273</v>
       </c>
       <c r="AF9" s="9"/>
       <c r="AG9" s="5">
         <v>0</v>
       </c>
       <c r="AH9" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI9" s="11">
-        <v>4</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI9" s="11"/>
       <c r="AJ9" s="12">
-        <v>46154</v>
+        <v>46028</v>
       </c>
       <c t="s" r="AK9" s="4">
         <v>52</v>
@@ -1910,14 +1995,16 @@
       <c t="s" r="AQ9" s="4">
         <v>55</v>
       </c>
-      <c r="AR9" s="4"/>
+      <c t="s" r="AR9" s="4">
+        <v>67</v>
+      </c>
       <c t="s" r="AS9" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="10" ht="13.5" customHeight="1">
+    <row r="10" ht="24.75" customHeight="1">
       <c r="A10" s="2">
-        <v>19518</v>
+        <v>19666</v>
       </c>
       <c r="B10" s="3">
         <v>0</v>
@@ -1925,9 +2012,7 @@
       <c t="s" r="C10" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D10" s="4">
-        <v>45</v>
-      </c>
+      <c r="D10" s="4"/>
       <c t="s" r="E10" s="4">
         <v>46</v>
       </c>
@@ -1957,68 +2042,66 @@
         <v>52</v>
       </c>
       <c r="O10" s="5">
-        <v>63298.069999999992</v>
+        <v>31623.699999999997</v>
       </c>
       <c r="P10" s="5">
-        <v>63298.069999999992</v>
+        <v>31623.699999999997</v>
       </c>
       <c r="Q10" s="6">
-        <v>0.059577880093305779</v>
+        <v>-0.1014171624585215</v>
       </c>
       <c r="R10" s="7">
-        <v>676</v>
+        <v>293</v>
       </c>
       <c r="S10" s="6">
-        <v>0.016541353383458635</v>
+        <v>-0.16045845272206305</v>
       </c>
       <c r="T10" s="6">
-        <v>0.33963196824168573</v>
+        <v>0.26282438487590004</v>
       </c>
       <c r="U10" s="6">
-        <v>0.000241525531505147</v>
+        <v>-0.058070703301637695</v>
       </c>
       <c r="V10" s="6">
-        <v>0.021292908298783834</v>
+        <v>0.029054474966559888</v>
       </c>
       <c r="W10" s="6">
-        <v>-0.0046574879771215773</v>
+        <v>0.0058377103248512989</v>
       </c>
       <c r="X10" s="8">
-        <v>24.717295417789757</v>
+        <v>22.501484653465347</v>
       </c>
       <c r="Y10" s="6">
-        <v>0.83378016085790885</v>
+        <v>0.97029702970297027</v>
       </c>
       <c r="Z10" s="6">
-        <v>0.0215633423180593</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="8">
-        <v>6.2278286149162856</v>
+        <v>3.3255402730375425</v>
       </c>
       <c r="AB10" s="8">
-        <v>4.7264117486338799</v>
+        <v>3.1315</v>
       </c>
       <c r="AC10" s="8">
-        <v>11.453355</v>
+        <v>6.313879</v>
       </c>
       <c r="AD10" s="8">
-        <v>18.464195687331536</v>
+        <v>14.409818811881188</v>
       </c>
       <c r="AE10" s="6">
-        <v>0.7978436657681941</v>
+        <v>0.97524752475247523</v>
       </c>
       <c r="AF10" s="9"/>
       <c r="AG10" s="5">
-        <v>-2155.6999999999998</v>
+        <v>0</v>
       </c>
       <c r="AH10" s="10">
         <v>5</v>
       </c>
-      <c r="AI10" s="11">
-        <v>5</v>
-      </c>
+      <c r="AI10" s="11"/>
       <c r="AJ10" s="12">
-        <v>45939</v>
+        <v>46020</v>
       </c>
       <c t="s" r="AK10" s="4">
         <v>52</v>
@@ -2041,14 +2124,16 @@
       <c t="s" r="AQ10" s="4">
         <v>55</v>
       </c>
-      <c r="AR10" s="4"/>
+      <c t="s" r="AR10" s="4">
+        <v>68</v>
+      </c>
       <c t="s" r="AS10" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" ht="13.5" customHeight="1">
       <c r="A11" s="2">
-        <v>19519</v>
+        <v>19691</v>
       </c>
       <c r="B11" s="3">
         <v>0</v>
@@ -2056,11 +2141,9 @@
       <c t="s" r="C11" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D11" s="4">
-        <v>45</v>
-      </c>
+      <c r="D11" s="4"/>
       <c t="s" r="E11" s="4">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c t="s" r="F11" s="4">
         <v>47</v>
@@ -2088,68 +2171,66 @@
         <v>52</v>
       </c>
       <c r="O11" s="5">
-        <v>67649.889999999999</v>
+        <v>36387.289999999994</v>
       </c>
       <c r="P11" s="5">
-        <v>67649.889999999999</v>
+        <v>36387.289999999994</v>
       </c>
       <c r="Q11" s="6">
-        <v>-0.19878833860290246</v>
+        <v>-0.070231971275463989</v>
       </c>
       <c r="R11" s="7">
-        <v>764</v>
+        <v>335</v>
       </c>
       <c r="S11" s="6">
-        <v>-0.09155766944114152</v>
+        <v>-0.12073490813648291</v>
       </c>
       <c r="T11" s="6">
-        <v>0.31200488130875009</v>
+        <v>0.30466604135674846</v>
       </c>
       <c r="U11" s="6">
-        <v>0.011464111767217951</v>
+        <v>-0.013839678635039871</v>
       </c>
       <c r="V11" s="6">
-        <v>0.018386349186968375</v>
+        <v>0.03901626089769257</v>
       </c>
       <c r="W11" s="6">
-        <v>-0.00097510136380118289</v>
+        <v>0.015869991966975281</v>
       </c>
       <c r="X11" s="8">
-        <v>23.661255924170614</v>
+        <v>27.566158883248733</v>
       </c>
       <c r="Y11" s="6">
-        <v>0.60663507109004744</v>
+        <v>0.82741116751269039</v>
       </c>
       <c r="Z11" s="6">
-        <v>0.035545023696682464</v>
+        <v>0.076142131979695438</v>
       </c>
       <c r="AA11" s="8">
-        <v>7.182227958387517</v>
+        <v>3.2623653958944279</v>
       </c>
       <c r="AB11" s="8">
-        <v>3.6947619047619047</v>
+        <v>8.3521260204081624</v>
       </c>
       <c r="AC11" s="8">
-        <v>11.176833999999999</v>
+        <v>12.408906999999999</v>
       </c>
       <c r="AD11" s="8">
-        <v>17.995773933649289</v>
+        <v>18.123265482233503</v>
       </c>
       <c r="AE11" s="6">
-        <v>0.80568720379146919</v>
+        <v>0.7208121827411168</v>
       </c>
       <c r="AF11" s="9"/>
       <c r="AG11" s="5">
-        <v>-884.70000000000005</v>
+        <v>91.890000000000001</v>
       </c>
       <c r="AH11" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI11" s="11">
-        <v>4</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AI11" s="11"/>
       <c r="AJ11" s="12">
-        <v>46036</v>
+        <v>45954</v>
       </c>
       <c t="s" r="AK11" s="4">
         <v>52</v>
@@ -2172,24 +2253,24 @@
       <c t="s" r="AQ11" s="4">
         <v>55</v>
       </c>
-      <c r="AR11" s="4"/>
+      <c t="s" r="AR11" s="4">
+        <v>56</v>
+      </c>
       <c t="s" r="AS11" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" ht="13.5" customHeight="1">
       <c r="A12" s="2">
-        <v>19526</v>
+        <v>19693</v>
       </c>
       <c r="B12" s="3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c t="s" r="C12" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D12" s="4">
-        <v>45</v>
-      </c>
+      <c r="D12" s="4"/>
       <c t="s" r="E12" s="4">
         <v>46</v>
       </c>
@@ -2219,68 +2300,66 @@
         <v>52</v>
       </c>
       <c r="O12" s="5">
-        <v>27510.899999999998</v>
+        <v>2651.48</v>
       </c>
       <c r="P12" s="5">
-        <v>27510.899999999998</v>
+        <v>2651.48</v>
       </c>
       <c r="Q12" s="6">
-        <v>0.37382771535580517</v>
+        <v>-0.45279650645649272</v>
       </c>
       <c r="R12" s="7">
-        <v>262</v>
+        <v>24</v>
       </c>
       <c r="S12" s="6">
-        <v>0.24761904761904763</v>
+        <v>-0.51020408163265307</v>
       </c>
       <c r="T12" s="6">
-        <v>0.34462039409833917</v>
+        <v>0</v>
       </c>
       <c r="U12" s="6">
-        <v>0.014659542217811848</v>
+        <v>-0.31269328827673604</v>
       </c>
       <c r="V12" s="6">
-        <v>0.022895979411796778</v>
+        <v>0.035339508500912699</v>
       </c>
       <c r="W12" s="6">
-        <v>-0.014870142379929409</v>
+        <v>-0.0031672877034712686</v>
       </c>
       <c r="X12" s="8">
-        <v>22.771098936170212</v>
+        <v>30.314816666666665</v>
       </c>
       <c r="Y12" s="6">
-        <v>0.84042553191489366</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="Z12" s="6">
-        <v>0.0053191489361702126</v>
+        <v>0.055555555555555552</v>
       </c>
       <c r="AA12" s="8">
-        <v>3.6611107142857144</v>
+        <v>3.597826086956522</v>
       </c>
       <c r="AB12" s="8">
-        <v>3.8667553191489366</v>
+        <v>6.7101833333333332</v>
       </c>
       <c r="AC12" s="8">
-        <v>7.8051250000000003</v>
+        <v>10.444444000000001</v>
       </c>
       <c r="AD12" s="8">
-        <v>13.682535638297871</v>
+        <v>18.652777777777779</v>
       </c>
       <c r="AE12" s="6">
-        <v>0.92021276595744683</v>
+        <v>0.5</v>
       </c>
       <c r="AF12" s="9"/>
       <c r="AG12" s="5">
-        <v>-187.03</v>
+        <v>0</v>
       </c>
       <c r="AH12" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI12" s="11">
-        <v>3</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI12" s="11"/>
       <c r="AJ12" s="12">
-        <v>46043</v>
+        <v>46015</v>
       </c>
       <c t="s" r="AK12" s="4">
         <v>52</v>
@@ -2303,14 +2382,16 @@
       <c t="s" r="AQ12" s="4">
         <v>55</v>
       </c>
-      <c r="AR12" s="4"/>
+      <c t="s" r="AR12" s="4">
+        <v>70</v>
+      </c>
       <c t="s" r="AS12" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="2">
-        <v>19560</v>
+        <v>19700</v>
       </c>
       <c r="B13" s="3">
         <v>0</v>
@@ -2319,10 +2400,10 @@
         <v>44</v>
       </c>
       <c t="s" r="D13" s="4">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c t="s" r="E13" s="4">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c t="s" r="F13" s="4">
         <v>47</v>
@@ -2350,68 +2431,66 @@
         <v>52</v>
       </c>
       <c r="O13" s="5">
-        <v>69312.48000000001</v>
+        <v>21880.779999999999</v>
       </c>
       <c r="P13" s="5">
-        <v>69312.48000000001</v>
+        <v>21880.779999999999</v>
       </c>
       <c r="Q13" s="6">
-        <v>0.45816391102972864</v>
+        <v>-0.092004320710236454</v>
       </c>
       <c r="R13" s="7">
-        <v>801</v>
+        <v>247</v>
       </c>
       <c r="S13" s="6">
-        <v>0.69344608879492609</v>
+        <v>-0.1453287197231834</v>
       </c>
       <c r="T13" s="6">
-        <v>0.26184861369842777</v>
+        <v>0</v>
       </c>
       <c r="U13" s="6">
-        <v>-0.040814485356749607</v>
+        <v>-0.34349689544888251</v>
       </c>
       <c r="V13" s="6">
-        <v>0.042860153034489611</v>
+        <v>0.033818218546139582</v>
       </c>
       <c r="W13" s="6">
-        <v>0.021139245053704618</v>
+        <v>0.022750057356273407</v>
       </c>
       <c r="X13" s="8">
-        <v>37.511748524590168</v>
+        <v>31.396865811965814</v>
       </c>
       <c r="Y13" s="6">
-        <v>0.70163934426229513</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="Z13" s="6">
-        <v>0.31147540983606559</v>
+        <v>0.20512820512820512</v>
       </c>
       <c r="AA13" s="8">
-        <v>21.540062767295598</v>
+        <v>8.3033203125000004</v>
       </c>
       <c r="AB13" s="8">
-        <v>3.5343385150812066</v>
+        <v>5.0008937500000004</v>
       </c>
       <c r="AC13" s="8">
-        <v>18.163694</v>
+        <v>11.330673000000001</v>
       </c>
       <c r="AD13" s="8">
-        <v>31.791202131147543</v>
+        <v>20.366666666666667</v>
       </c>
       <c r="AE13" s="6">
-        <v>0.51475409836065578</v>
+        <v>0.54700854700854706</v>
       </c>
       <c r="AF13" s="9"/>
       <c r="AG13" s="5">
-        <v>-108.8</v>
+        <v>-312.10000000000002</v>
       </c>
       <c r="AH13" s="10">
-        <v>4</v>
-      </c>
-      <c r="AI13" s="11">
-        <v>4</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI13" s="11"/>
       <c r="AJ13" s="12">
-        <v>46037</v>
+        <v>45938</v>
       </c>
       <c t="s" r="AK13" s="4">
         <v>52</v>
@@ -2435,15 +2514,15 @@
         <v>55</v>
       </c>
       <c t="s" r="AR13" s="4">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c t="s" r="AS13" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" ht="13.5" customHeight="1">
       <c r="A14" s="2">
-        <v>19561</v>
+        <v>19722</v>
       </c>
       <c r="B14" s="3">
         <v>0</v>
@@ -2451,11 +2530,9 @@
       <c t="s" r="C14" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D14" s="4">
-        <v>58</v>
-      </c>
+      <c r="D14" s="4"/>
       <c t="s" r="E14" s="4">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c t="s" r="F14" s="4">
         <v>47</v>
@@ -2483,68 +2560,66 @@
         <v>52</v>
       </c>
       <c r="O14" s="5">
-        <v>21569.470000000001</v>
+        <v>18735.23</v>
       </c>
       <c r="P14" s="5">
-        <v>21569.470000000001</v>
+        <v>18735.23</v>
       </c>
       <c r="Q14" s="6">
-        <v>0.18429564523187136</v>
+        <v>-0.17404564537610112</v>
       </c>
       <c r="R14" s="7">
-        <v>221</v>
+        <v>174</v>
       </c>
       <c r="S14" s="6">
-        <v>0.27745664739884401</v>
+        <v>-0.26890756302521013</v>
       </c>
       <c r="T14" s="6">
-        <v>0.31792812248052454</v>
+        <v>0</v>
       </c>
       <c r="U14" s="6">
-        <v>-0.0012503274303911965</v>
+        <v>-0.31037569327945269</v>
       </c>
       <c r="V14" s="6">
-        <v>0.063464424485163512</v>
+        <v>0.016621012925915508</v>
       </c>
       <c r="W14" s="6">
-        <v>0.014677875719709384</v>
+        <v>-0.013791744216644258</v>
       </c>
       <c r="X14" s="8">
-        <v>24.309150326797386</v>
+        <v>28.39626261682243</v>
       </c>
       <c r="Y14" s="6">
-        <v>0.65359477124183007</v>
+        <v>0.58878504672897192</v>
       </c>
       <c r="Z14" s="6">
-        <v>0</v>
+        <v>0.12149532710280374</v>
       </c>
       <c r="AA14" s="8">
-        <v>4.0860066037735852</v>
+        <v>3.5352488505747126</v>
       </c>
       <c r="AB14" s="8">
-        <v>2.6816881578947367</v>
+        <v>10.642307692307693</v>
       </c>
       <c r="AC14" s="8">
-        <v>6.5601070000000004</v>
+        <v>14.096730000000001</v>
       </c>
       <c r="AD14" s="8">
-        <v>13.502832026143793</v>
+        <v>19.903271028037384</v>
       </c>
       <c r="AE14" s="6">
-        <v>0.85620915032679734</v>
+        <v>0.62616822429906538</v>
       </c>
       <c r="AF14" s="9"/>
       <c r="AG14" s="5">
-        <v>0</v>
+        <v>-51.899999999999999</v>
       </c>
       <c r="AH14" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI14" s="11">
-        <v>4</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI14" s="11"/>
       <c r="AJ14" s="12">
-        <v>46034</v>
+        <v>45937</v>
       </c>
       <c t="s" r="AK14" s="4">
         <v>52</v>
@@ -2568,27 +2643,25 @@
         <v>55</v>
       </c>
       <c t="s" r="AR14" s="4">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c t="s" r="AS14" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" ht="13.5" customHeight="1">
       <c r="A15" s="2">
-        <v>19562</v>
+        <v>19730</v>
       </c>
       <c r="B15" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="s" r="C15" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D15" s="4">
-        <v>58</v>
-      </c>
+      <c r="D15" s="4"/>
       <c t="s" r="E15" s="4">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c t="s" r="F15" s="4">
         <v>47</v>
@@ -2616,68 +2689,66 @@
         <v>52</v>
       </c>
       <c r="O15" s="5">
-        <v>11350.85</v>
+        <v>33666.540000000001</v>
       </c>
       <c r="P15" s="5">
-        <v>11350.85</v>
+        <v>33666.540000000001</v>
       </c>
       <c r="Q15" s="6">
-        <v>0.14218597017658796</v>
+        <v>-0.092723634135206789</v>
       </c>
       <c r="R15" s="7">
-        <v>137</v>
+        <v>322</v>
       </c>
       <c r="S15" s="6">
-        <v>0.52222222222222214</v>
+        <v>-0.18274111675126903</v>
       </c>
       <c r="T15" s="6">
-        <v>0.32145141553275741</v>
+        <v>0.61462456492410567</v>
       </c>
       <c r="U15" s="6">
-        <v>0.0018127981604901834</v>
+        <v>0.27235624747895087</v>
       </c>
       <c r="V15" s="6">
-        <v>0.10026139011615869</v>
+        <v>0.015035343697332722</v>
       </c>
       <c r="W15" s="6">
-        <v>0.047512036543518765</v>
+        <v>4.2118970348601308E-05</v>
       </c>
       <c r="X15" s="8">
-        <v>29.620067346938775</v>
+        <v>28.14620396039604</v>
       </c>
       <c r="Y15" s="6">
-        <v>1</v>
+        <v>0.60396039603960394</v>
       </c>
       <c r="Z15" s="6">
-        <v>0.12244897959183673</v>
+        <v>0.15841584158415842</v>
       </c>
       <c r="AA15" s="8">
-        <v>5.0946564885496182</v>
+        <v>5.6400105590062113</v>
       </c>
       <c r="AB15" s="8">
-        <v>7.0661400000000008</v>
+        <v>8.4825009999999992</v>
       </c>
       <c r="AC15" s="8">
-        <v>11.847754999999999</v>
+        <v>16.628682999999999</v>
       </c>
       <c r="AD15" s="8">
-        <v>18.254081632653062</v>
+        <v>22.361055445544558</v>
       </c>
       <c r="AE15" s="6">
-        <v>0.65306122448979587</v>
+        <v>0.6633663366336634</v>
       </c>
       <c r="AF15" s="9"/>
       <c r="AG15" s="5">
         <v>0</v>
       </c>
       <c r="AH15" s="10">
-        <v>4</v>
-      </c>
-      <c r="AI15" s="11">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI15" s="11"/>
       <c r="AJ15" s="12">
-        <v>46036</v>
+        <v>45982</v>
       </c>
       <c t="s" r="AK15" s="4">
         <v>52</v>
@@ -2700,14 +2771,16 @@
       <c t="s" r="AQ15" s="4">
         <v>55</v>
       </c>
-      <c r="AR15" s="4"/>
+      <c t="s" r="AR15" s="4">
+        <v>74</v>
+      </c>
       <c t="s" r="AS15" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" ht="13.5" customHeight="1">
       <c r="A16" s="2">
-        <v>19635</v>
+        <v>19752</v>
       </c>
       <c r="B16" s="3">
         <v>0</v>
@@ -2715,11 +2788,9 @@
       <c t="s" r="C16" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D16" s="4">
-        <v>45</v>
-      </c>
+      <c r="D16" s="4"/>
       <c t="s" r="E16" s="4">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c t="s" r="F16" s="4">
         <v>47</v>
@@ -2747,68 +2818,66 @@
         <v>52</v>
       </c>
       <c r="O16" s="5">
-        <v>23857.549999999999</v>
+        <v>12449.93</v>
       </c>
       <c r="P16" s="5">
-        <v>23857.549999999999</v>
+        <v>12449.93</v>
       </c>
       <c r="Q16" s="6">
-        <v>0.043980327745466674</v>
+        <v>0.11910992058319891</v>
       </c>
       <c r="R16" s="7">
-        <v>261</v>
+        <v>138</v>
       </c>
       <c r="S16" s="6">
-        <v>-0.0076045627376425395</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="T16" s="6">
-        <v>0.37540952025669022</v>
+        <v>1.6064347349744136E-06</v>
       </c>
       <c r="U16" s="6">
-        <v>0.025058792709226223</v>
+        <v>-0.32791509671138713</v>
       </c>
       <c r="V16" s="6">
-        <v>0.040571580065849176</v>
+        <v>0.033017053107929122</v>
       </c>
       <c r="W16" s="6">
-        <v>0.0049677565382866221</v>
+        <v>-0.04800187631577045</v>
       </c>
       <c r="X16" s="8">
-        <v>21.840350877192982</v>
+        <v>38.318094285714288</v>
       </c>
       <c r="Y16" s="6">
-        <v>0.73684210526315785</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="Z16" s="6">
-        <v>0.017543859649122806</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="AA16" s="8">
-        <v>5.270849800796813</v>
+        <v>7.0509528571428577</v>
       </c>
       <c r="AB16" s="8">
-        <v>4.182504968944099</v>
+        <v>18.095322807017542</v>
       </c>
       <c r="AC16" s="8">
-        <v>8.7307330000000007</v>
+        <v>27.495698999999998</v>
       </c>
       <c r="AD16" s="8">
-        <v>16.091130409356722</v>
+        <v>28.981665714285715</v>
       </c>
       <c r="AE16" s="6">
-        <v>0.88888888888888884</v>
+        <v>0.44285714285714284</v>
       </c>
       <c r="AF16" s="9"/>
       <c r="AG16" s="5">
-        <v>-465.30000000000001</v>
+        <v>-194.59999999999999</v>
       </c>
       <c r="AH16" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI16" s="11">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI16" s="11"/>
       <c r="AJ16" s="12">
-        <v>45975</v>
+        <v>44781</v>
       </c>
       <c t="s" r="AK16" s="4">
         <v>52</v>
@@ -2831,14 +2900,16 @@
       <c t="s" r="AQ16" s="4">
         <v>55</v>
       </c>
-      <c r="AR16" s="4"/>
+      <c t="s" r="AR16" s="4">
+        <v>76</v>
+      </c>
       <c t="s" r="AS16" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" ht="13.5" customHeight="1">
       <c r="A17" s="2">
-        <v>19665</v>
+        <v>19754</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
@@ -2850,7 +2921,7 @@
         <v>45</v>
       </c>
       <c t="s" r="E17" s="4">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c t="s" r="F17" s="4">
         <v>47</v>
@@ -2878,68 +2949,66 @@
         <v>52</v>
       </c>
       <c r="O17" s="5">
-        <v>26490.529999999999</v>
+        <v>38694.610000000001</v>
       </c>
       <c r="P17" s="5">
-        <v>26490.529999999999</v>
+        <v>38694.610000000001</v>
       </c>
       <c r="Q17" s="6">
-        <v>0.22542684385117728</v>
+        <v>-0.12293475629602968</v>
       </c>
       <c r="R17" s="7">
-        <v>296</v>
+        <v>377</v>
       </c>
       <c r="S17" s="6">
-        <v>0.18875502008032119</v>
+        <v>-0.14512471655328796</v>
       </c>
       <c r="T17" s="6">
-        <v>0.35327432482475818</v>
+        <v>0.30667290095442229</v>
       </c>
       <c r="U17" s="6">
-        <v>0.0039143837439266039</v>
+        <v>-0.029691259325265194</v>
       </c>
       <c r="V17" s="6">
-        <v>0.019988105183248506</v>
+        <v>0.021231949359355219</v>
       </c>
       <c r="W17" s="6">
-        <v>-0.0074809564021557891</v>
+        <v>0.0012175339149302707</v>
       </c>
       <c r="X17" s="8">
-        <v>31.460621078431373</v>
+        <v>22.016830541871919</v>
       </c>
       <c r="Y17" s="6">
-        <v>0.92156862745098034</v>
+        <v>0.9211822660098522</v>
       </c>
       <c r="Z17" s="6">
-        <v>0.2107843137254902</v>
+        <v>0.0049261083743842365</v>
       </c>
       <c r="AA17" s="8">
-        <v>9.7701034364261172</v>
+        <v>2.2779981481481482</v>
       </c>
       <c r="AB17" s="8">
-        <v>5.2954314720812183</v>
+        <v>4.7286064676616917</v>
       </c>
       <c r="AC17" s="8">
-        <v>12.567868000000001</v>
+        <v>7.5808179999999998</v>
       </c>
       <c r="AD17" s="8">
-        <v>23.07916617647059</v>
+        <v>14.910591133004926</v>
       </c>
       <c r="AE17" s="6">
-        <v>0.6029411764705882</v>
+        <v>0.91625615763546797</v>
       </c>
       <c r="AF17" s="9"/>
       <c r="AG17" s="5">
-        <v>-568.63</v>
+        <v>0</v>
       </c>
       <c r="AH17" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI17" s="11">
-        <v>3</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="AI17" s="11"/>
       <c r="AJ17" s="12">
-        <v>46038</v>
+        <v>45989</v>
       </c>
       <c t="s" r="AK17" s="4">
         <v>52</v>
@@ -2962,24 +3031,28 @@
       <c t="s" r="AQ17" s="4">
         <v>55</v>
       </c>
-      <c r="AR17" s="4"/>
+      <c t="s" r="AR17" s="4">
+        <v>56</v>
+      </c>
       <c t="s" r="AS17" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" ht="13.5" customHeight="1">
       <c r="A18" s="2">
-        <v>19704</v>
+        <v>19755</v>
       </c>
       <c r="B18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C18" s="4">
         <v>44</v>
       </c>
-      <c r="D18" s="4"/>
+      <c t="s" r="D18" s="4">
+        <v>45</v>
+      </c>
       <c t="s" r="E18" s="4">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c t="s" r="F18" s="4">
         <v>47</v>
@@ -3007,68 +3080,66 @@
         <v>52</v>
       </c>
       <c r="O18" s="5">
-        <v>29124.019999999997</v>
+        <v>11491.5</v>
       </c>
       <c r="P18" s="5">
-        <v>29124.019999999997</v>
+        <v>11491.5</v>
       </c>
       <c r="Q18" s="6">
-        <v>0.17396321955281868</v>
+        <v>-0.3870837153559491</v>
       </c>
       <c r="R18" s="7">
-        <v>322</v>
+        <v>124</v>
       </c>
       <c r="S18" s="6">
-        <v>0.23371647509578541</v>
+        <v>-0.35416666666666663</v>
       </c>
       <c r="T18" s="6">
-        <v>0.28684683982499665</v>
+        <v>0.0010425096810686161</v>
       </c>
       <c r="U18" s="6">
-        <v>-0.031797014972520965</v>
+        <v>-0.33716399077579079</v>
       </c>
       <c r="V18" s="6">
-        <v>0.05754646851636553</v>
+        <v>0.053332463124918419</v>
       </c>
       <c r="W18" s="6">
-        <v>0.025159456009163569</v>
+        <v>0.0071243962929121527</v>
       </c>
       <c r="X18" s="8">
-        <v>23.212040569395018</v>
+        <v>29.593137254901961</v>
       </c>
       <c r="Y18" s="6">
-        <v>0.72241992882562278</v>
+        <v>1</v>
       </c>
       <c r="Z18" s="6">
-        <v>0.02491103202846975</v>
+        <v>0.078431372549019607</v>
       </c>
       <c r="AA18" s="8">
-        <v>3.2468006191950463</v>
+        <v>5.2997306451612909</v>
       </c>
       <c r="AB18" s="8">
-        <v>2.2318127737226279</v>
+        <v>5.9276679999999997</v>
       </c>
       <c r="AC18" s="8">
-        <v>5.4139629999999999</v>
+        <v>10.342708</v>
       </c>
       <c r="AD18" s="8">
-        <v>12.199288612099645</v>
+        <v>19.028105882352943</v>
       </c>
       <c r="AE18" s="6">
-        <v>0.89679715302491103</v>
+        <v>0.52941176470588236</v>
       </c>
       <c r="AF18" s="9"/>
       <c r="AG18" s="5">
         <v>0</v>
       </c>
       <c r="AH18" s="10">
-        <v>3</v>
-      </c>
-      <c r="AI18" s="11">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI18" s="11"/>
       <c r="AJ18" s="12">
-        <v>45783</v>
+        <v>45986</v>
       </c>
       <c t="s" r="AK18" s="4">
         <v>52</v>
@@ -3091,14 +3162,16 @@
       <c t="s" r="AQ18" s="4">
         <v>55</v>
       </c>
-      <c r="AR18" s="4"/>
+      <c t="s" r="AR18" s="4">
+        <v>67</v>
+      </c>
       <c t="s" r="AS18" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" ht="13.5" customHeight="1">
       <c r="A19" s="2">
-        <v>19714</v>
+        <v>19762</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
@@ -3107,10 +3180,10 @@
         <v>44</v>
       </c>
       <c t="s" r="D19" s="4">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c t="s" r="E19" s="4">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c t="s" r="F19" s="4">
         <v>47</v>
@@ -3128,78 +3201,76 @@
         <v>47</v>
       </c>
       <c t="s" r="K19" s="4">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c t="s" r="L19" s="4">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="M19" s="4"/>
       <c t="s" r="N19" s="4">
         <v>52</v>
       </c>
       <c r="O19" s="5">
-        <v>40124.410000000003</v>
+        <v>14657.349999999999</v>
       </c>
       <c r="P19" s="5">
-        <v>40124.410000000003</v>
+        <v>14657.349999999999</v>
       </c>
       <c r="Q19" s="6">
-        <v>0.021649874866738195</v>
+        <v>-0.09446286873639298</v>
       </c>
       <c r="R19" s="7">
-        <v>414</v>
+        <v>186</v>
       </c>
       <c r="S19" s="6">
-        <v>0.089473684210526372</v>
+        <v>-0.097087378640776656</v>
       </c>
       <c r="T19" s="6">
-        <v>0.30309587854375925</v>
+        <v>-0.00067761225596714273</v>
       </c>
       <c r="U19" s="6">
-        <v>0.0044664407526490727</v>
+        <v>-0.33968022869072512</v>
       </c>
       <c r="V19" s="6">
-        <v>0.020123062245650466</v>
+        <v>0.056447754880657147</v>
       </c>
       <c r="W19" s="6">
-        <v>-0.0095474051830294823</v>
+        <v>-0.012686843119663513</v>
       </c>
       <c r="X19" s="8">
-        <v>23.40478454258675</v>
+        <v>25.269952112676055</v>
       </c>
       <c r="Y19" s="6">
-        <v>0.65408805031446537</v>
+        <v>0.81690140845070425</v>
       </c>
       <c r="Z19" s="6">
-        <v>0.012618296529968454</v>
+        <v>0.028169014084507043</v>
       </c>
       <c r="AA19" s="8">
-        <v>4.4626216019417475</v>
+        <v>6.5098041176470591</v>
       </c>
       <c r="AB19" s="8">
-        <v>4.7461584415584417</v>
+        <v>6.8014070422535209</v>
       </c>
       <c r="AC19" s="8">
-        <v>8.6506570000000007</v>
+        <v>13.227143999999999</v>
       </c>
       <c r="AD19" s="8">
-        <v>16.00294447949527</v>
+        <v>20.293191549295777</v>
       </c>
       <c r="AE19" s="6">
-        <v>0.83280757097791802</v>
+        <v>0.77464788732394363</v>
       </c>
       <c r="AF19" s="9"/>
       <c r="AG19" s="5">
-        <v>-333.60000000000002</v>
+        <v>-3048.0999999999999</v>
       </c>
       <c r="AH19" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI19" s="11">
         <v>2</v>
       </c>
+      <c r="AI19" s="11"/>
       <c r="AJ19" s="12">
-        <v>46156</v>
+        <v>46119</v>
       </c>
       <c t="s" r="AK19" s="4">
         <v>52</v>
@@ -3222,14 +3293,16 @@
       <c t="s" r="AQ19" s="4">
         <v>55</v>
       </c>
-      <c r="AR19" s="4"/>
+      <c t="s" r="AR19" s="4">
+        <v>80</v>
+      </c>
       <c t="s" r="AS19" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" ht="13.5" customHeight="1">
       <c r="A20" s="2">
-        <v>19748</v>
+        <v>19787</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
@@ -3237,11 +3310,9 @@
       <c t="s" r="C20" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D20" s="4">
-        <v>58</v>
-      </c>
+      <c r="D20" s="4"/>
       <c t="s" r="E20" s="4">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c t="s" r="F20" s="4">
         <v>47</v>
@@ -3269,68 +3340,66 @@
         <v>52</v>
       </c>
       <c r="O20" s="5">
-        <v>26595.790000000001</v>
+        <v>11438.700000000001</v>
       </c>
       <c r="P20" s="5">
-        <v>26595.790000000001</v>
+        <v>11438.700000000001</v>
       </c>
       <c r="Q20" s="6">
-        <v>0.41789841655386528</v>
+        <v>0.63861086161475944</v>
       </c>
       <c r="R20" s="7">
-        <v>315</v>
+        <v>128</v>
       </c>
       <c r="S20" s="6">
-        <v>0.35775862068965525</v>
+        <v>0.47126436781609193</v>
       </c>
       <c r="T20" s="6">
-        <v>0.33316816308145014</v>
+        <v>0</v>
       </c>
       <c r="U20" s="6">
-        <v>0.015736719984629145</v>
+        <v>-0.35097344978013234</v>
       </c>
       <c r="V20" s="6">
-        <v>0.045587835518328276</v>
+        <v>0.024455925935639541</v>
       </c>
       <c r="W20" s="6">
-        <v>0.0061319667511286558</v>
+        <v>-0.01916441553673057</v>
       </c>
       <c r="X20" s="8">
-        <v>21.822863461538461</v>
+        <v>25.769736842105264</v>
       </c>
       <c r="Y20" s="6">
-        <v>0.91025641025641024</v>
+        <v>1</v>
       </c>
       <c r="Z20" s="6">
-        <v>0.019230769230769232</v>
+        <v>0.026315789473684209</v>
       </c>
       <c r="AA20" s="8">
-        <v>3.418201644736842</v>
+        <v>6.8309881481481485</v>
       </c>
       <c r="AB20" s="8">
-        <v>4.6882032467532468</v>
+        <v>4.451852777777777</v>
       </c>
       <c r="AC20" s="8">
-        <v>7.2802600000000002</v>
+        <v>12.276541999999999</v>
       </c>
       <c r="AD20" s="8">
-        <v>14.708333333333334</v>
+        <v>18.045176315789472</v>
       </c>
       <c r="AE20" s="6">
-        <v>0.92948717948717952</v>
+        <v>0.76315789473684215</v>
       </c>
       <c r="AF20" s="9"/>
       <c r="AG20" s="5">
-        <v>-327.10000000000002</v>
+        <v>-1016.8</v>
       </c>
       <c r="AH20" s="10">
-        <v>4</v>
-      </c>
-      <c r="AI20" s="11">
-        <v>4</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="AI20" s="11"/>
       <c r="AJ20" s="12">
-        <v>46035</v>
+        <v>46036</v>
       </c>
       <c t="s" r="AK20" s="4">
         <v>52</v>
@@ -3353,26 +3422,26 @@
       <c t="s" r="AQ20" s="4">
         <v>55</v>
       </c>
-      <c r="AR20" s="4"/>
+      <c t="s" r="AR20" s="4">
+        <v>82</v>
+      </c>
       <c t="s" r="AS20" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" ht="13.5" customHeight="1">
       <c r="A21" s="2">
-        <v>19793</v>
+        <v>19794</v>
       </c>
       <c r="B21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C21" s="4">
         <v>44</v>
       </c>
-      <c t="s" r="D21" s="4">
-        <v>58</v>
-      </c>
+      <c r="D21" s="4"/>
       <c t="s" r="E21" s="4">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c t="s" r="F21" s="4">
         <v>47</v>
@@ -3400,68 +3469,66 @@
         <v>52</v>
       </c>
       <c r="O21" s="5">
-        <v>10802.15</v>
+        <v>37148.18</v>
       </c>
       <c r="P21" s="5">
-        <v>10802.15</v>
+        <v>37148.18</v>
       </c>
       <c r="Q21" s="6">
-        <v>0.1289577508948867</v>
+        <v>0.03825289949471089</v>
       </c>
       <c r="R21" s="7">
-        <v>123</v>
+        <v>359</v>
       </c>
       <c r="S21" s="6">
-        <v>0.14953271028037385</v>
+        <v>-0.0082872928176795924</v>
       </c>
       <c r="T21" s="6">
-        <v>0.36385789865906326</v>
+        <v>0</v>
       </c>
       <c r="U21" s="6">
-        <v>0.0540316140768273</v>
+        <v>-0.35916914368348596</v>
       </c>
       <c r="V21" s="6">
-        <v>0.10064454761320664</v>
+        <v>0.015225819945956974</v>
       </c>
       <c r="W21" s="6">
-        <v>0.036160162560231066</v>
+        <v>0.00047166509907080236</v>
       </c>
       <c r="X21" s="8">
-        <v>20.691349367088609</v>
+        <v>30.035585405405406</v>
       </c>
       <c r="Y21" s="6">
-        <v>0.94936708860759489</v>
+        <v>0.45945945945945948</v>
       </c>
       <c r="Z21" s="6">
-        <v>0.012658227848101266</v>
+        <v>0.15675675675675677</v>
       </c>
       <c r="AA21" s="8">
-        <v>4.6655737704918039</v>
+        <v>6.2813022160664822</v>
       </c>
       <c r="AB21" s="8">
-        <v>2.2779283783783781</v>
+        <v>8.6783245901639336</v>
       </c>
       <c r="AC21" s="8">
-        <v>6.6747139999999998</v>
+        <v>13.039531999999999</v>
       </c>
       <c r="AD21" s="8">
-        <v>14.229113924050631</v>
+        <v>23.59171135135135</v>
       </c>
       <c r="AE21" s="6">
-        <v>0.94936708860759489</v>
+        <v>0.572972972972973</v>
       </c>
       <c r="AF21" s="9"/>
       <c r="AG21" s="5">
-        <v>-7.6299999999999999</v>
+        <v>-238.90000000000001</v>
       </c>
       <c r="AH21" s="10">
-        <v>4</v>
-      </c>
-      <c r="AI21" s="11">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI21" s="11"/>
       <c r="AJ21" s="12">
-        <v>45784</v>
+        <v>46155</v>
       </c>
       <c t="s" r="AK21" s="4">
         <v>52</v>
@@ -3485,15 +3552,15 @@
         <v>55</v>
       </c>
       <c t="s" r="AR21" s="4">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c t="s" r="AS21" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" ht="13.5" customHeight="1">
       <c r="A22" s="2">
-        <v>19844</v>
+        <v>19868</v>
       </c>
       <c r="B22" s="3">
         <v>0</v>
@@ -3502,10 +3569,10 @@
         <v>44</v>
       </c>
       <c t="s" r="D22" s="4">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c t="s" r="E22" s="4">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c t="s" r="F22" s="4">
         <v>47</v>
@@ -3533,66 +3600,62 @@
         <v>52</v>
       </c>
       <c r="O22" s="5">
-        <v>24959.080000000002</v>
+        <v>15927.4</v>
       </c>
       <c r="P22" s="5">
-        <v>24959.080000000002</v>
-      </c>
-      <c r="Q22" s="6"/>
+        <v>15927.4</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>0.10344875365451478</v>
+      </c>
       <c r="R22" s="7">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="S22" s="6">
-        <v>-0.31111111111111112</v>
+        <v>0</v>
       </c>
       <c r="T22" s="6">
-        <v>0.28846799240997661</v>
+        <v>0.15430481434509086</v>
       </c>
       <c r="U22" s="6">
-        <v>-0.038864585553634187</v>
+        <v>-0.16683674045983651</v>
       </c>
       <c r="V22" s="6">
-        <v>0.020899688610317362</v>
+        <v>0.022547277019475873</v>
       </c>
       <c r="W22" s="6">
-        <v>-0.010750917101111099</v>
+        <v>-0.017031687532177257</v>
       </c>
       <c r="X22" s="8">
-        <v>21.81777794871795</v>
+        <v>4.4667000000000003</v>
       </c>
       <c r="Y22" s="6">
-        <v>0.80512820512820515</v>
+        <v>1</v>
       </c>
       <c r="Z22" s="6">
-        <v>0.010256410256410256</v>
+        <v>0</v>
       </c>
       <c r="AA22" s="8">
-        <v>4.5836044715447155</v>
-      </c>
-      <c r="AB22" s="8">
-        <v>3.5343584615384613</v>
-      </c>
-      <c r="AC22" s="8">
-        <v>9.4560849999999999</v>
-      </c>
+        <v>13.234263959390864</v>
+      </c>
+      <c r="AB22" s="8"/>
+      <c r="AC22" s="8"/>
       <c r="AD22" s="8">
-        <v>14.290768717948719</v>
+        <v>0.4667</v>
       </c>
       <c r="AE22" s="6">
-        <v>0.94871794871794868</v>
+        <v>1</v>
       </c>
       <c r="AF22" s="9"/>
       <c r="AG22" s="5">
-        <v>0</v>
+        <v>-2013.0999999999999</v>
       </c>
       <c r="AH22" s="10">
-        <v>5</v>
-      </c>
-      <c r="AI22" s="11">
-        <v>4</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AI22" s="11"/>
       <c r="AJ22" s="12">
-        <v>46041</v>
+        <v>44781</v>
       </c>
       <c t="s" r="AK22" s="4">
         <v>52</v>
@@ -3615,17 +3678,19 @@
       <c t="s" r="AQ22" s="4">
         <v>55</v>
       </c>
-      <c r="AR22" s="4"/>
+      <c t="s" r="AR22" s="4">
+        <v>85</v>
+      </c>
       <c t="s" r="AS22" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" ht="13.5" customHeight="1">
       <c r="A23" s="2">
-        <v>19894</v>
+        <v>19881</v>
       </c>
       <c r="B23" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c t="s" r="C23" s="4">
         <v>44</v>
@@ -3634,7 +3699,7 @@
         <v>45</v>
       </c>
       <c t="s" r="E23" s="4">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c t="s" r="F23" s="4">
         <v>47</v>
@@ -3662,68 +3727,66 @@
         <v>52</v>
       </c>
       <c r="O23" s="5">
-        <v>35540.190000000002</v>
+        <v>23621.900000000001</v>
       </c>
       <c r="P23" s="5">
-        <v>35540.190000000002</v>
+        <v>23621.900000000001</v>
       </c>
       <c r="Q23" s="6">
-        <v>0.13111075819342788</v>
+        <v>-0.13173708820099139</v>
       </c>
       <c r="R23" s="7">
-        <v>380</v>
+        <v>218</v>
       </c>
       <c r="S23" s="6">
-        <v>0.043956043956044022</v>
+        <v>-0.10655737704918034</v>
       </c>
       <c r="T23" s="6">
-        <v>0.33191233361442352</v>
+        <v>129.12690067691423</v>
       </c>
       <c r="U23" s="6">
-        <v>-0.0024257776899898392</v>
+        <v>128.77746942879278</v>
       </c>
       <c r="V23" s="6">
-        <v>0.036144798325501354</v>
+        <v>0.029227623518853267</v>
       </c>
       <c r="W23" s="6">
-        <v>0.0052316265050918404</v>
+        <v>-0.0014570377488686344</v>
       </c>
       <c r="X23" s="8">
-        <v>22.915261685823758</v>
+        <v>20.297088554216867</v>
       </c>
       <c r="Y23" s="6">
-        <v>0.71647509578544066</v>
+        <v>0.85542168674698793</v>
       </c>
       <c r="Z23" s="6">
-        <v>0.019157088122605363</v>
+        <v>0.006024096385542169</v>
       </c>
       <c r="AA23" s="8">
-        <v>5.7236649171270715</v>
+        <v>2.1070171052631581</v>
       </c>
       <c r="AB23" s="8">
-        <v>3.7301284615384613</v>
+        <v>5.2307072727272725</v>
       </c>
       <c r="AC23" s="8">
-        <v>10.183914</v>
+        <v>7.3212520000000003</v>
       </c>
       <c r="AD23" s="8">
-        <v>16.429374329501918</v>
+        <v>13.557530722891565</v>
       </c>
       <c r="AE23" s="6">
-        <v>0.89272030651340994</v>
+        <v>0.94578313253012047</v>
       </c>
       <c r="AF23" s="9"/>
       <c r="AG23" s="5">
-        <v>-620.75999999999999</v>
+        <v>0</v>
       </c>
       <c r="AH23" s="10">
         <v>5</v>
       </c>
-      <c r="AI23" s="11">
-        <v>5</v>
-      </c>
+      <c r="AI23" s="11"/>
       <c r="AJ23" s="12">
-        <v>45978</v>
+        <v>46049</v>
       </c>
       <c t="s" r="AK23" s="4">
         <v>52</v>
@@ -3746,117 +3809,506 @@
       <c t="s" r="AQ23" s="4">
         <v>55</v>
       </c>
-      <c r="AR23" s="4"/>
+      <c t="s" r="AR23" s="4">
+        <v>87</v>
+      </c>
       <c t="s" r="AS23" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="24" ht="24.75" customHeight="1">
-      <c t="s" r="A24" s="13">
-        <v>64</v>
-      </c>
-      <c t="s" r="B24" s="13">
-        <v>65</v>
-      </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c t="s" r="N24" s="14">
-        <v>52</v>
-      </c>
-      <c t="s" r="O24" s="13">
-        <v>66</v>
-      </c>
-      <c t="s" r="P24" s="13">
+    <row r="24" ht="13.5" customHeight="1">
+      <c r="A24" s="2">
+        <v>19898</v>
+      </c>
+      <c r="B24" s="3">
+        <v>1</v>
+      </c>
+      <c t="s" r="C24" s="4">
+        <v>44</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c t="s" r="E24" s="4">
+        <v>88</v>
+      </c>
+      <c t="s" r="F24" s="4">
+        <v>47</v>
+      </c>
+      <c t="s" r="G24" s="4">
+        <v>48</v>
+      </c>
+      <c t="s" r="H24" s="4">
+        <v>49</v>
+      </c>
+      <c t="s" r="I24" s="4">
+        <v>50</v>
+      </c>
+      <c t="s" r="J24" s="4">
+        <v>47</v>
+      </c>
+      <c t="s" r="K24" s="4">
+        <v>51</v>
+      </c>
+      <c t="s" r="L24" s="4">
+        <v>51</v>
+      </c>
+      <c r="M24" s="4"/>
+      <c t="s" r="N24" s="4">
+        <v>52</v>
+      </c>
+      <c r="O24" s="5">
+        <v>9704.7999999999993</v>
+      </c>
+      <c r="P24" s="5">
+        <v>9704.7999999999993</v>
+      </c>
+      <c r="Q24" s="6">
+        <v>-0.13531352547202358</v>
+      </c>
+      <c r="R24" s="7">
+        <v>101</v>
+      </c>
+      <c r="S24" s="6">
+        <v>-0.24626865671641796</v>
+      </c>
+      <c r="T24" s="6">
+        <v>0.00572397164289836</v>
+      </c>
+      <c r="U24" s="6">
+        <v>-0.31514302200972716</v>
+      </c>
+      <c r="V24" s="6">
+        <v>0.020478629131975932</v>
+      </c>
+      <c r="W24" s="6">
+        <v>-0.035034106833731767</v>
+      </c>
+      <c r="X24" s="8">
+        <v>29.218433333333333</v>
+      </c>
+      <c r="Y24" s="6">
+        <v>0.68181818181818177</v>
+      </c>
+      <c r="Z24" s="6">
+        <v>0.07575757575757576</v>
+      </c>
+      <c r="AA24" s="8">
+        <v>3.7357365384615382</v>
+      </c>
+      <c r="AB24" s="8">
+        <v>10.643750000000001</v>
+      </c>
+      <c r="AC24" s="8">
+        <v>14.361642</v>
+      </c>
+      <c r="AD24" s="8">
+        <v>20.853284848484851</v>
+      </c>
+      <c r="AE24" s="6">
+        <v>0.56060606060606055</v>
+      </c>
+      <c r="AF24" s="9"/>
+      <c r="AG24" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="10">
+        <v>2</v>
+      </c>
+      <c r="AI24" s="11"/>
+      <c r="AJ24" s="12">
+        <v>45975</v>
+      </c>
+      <c t="s" r="AK24" s="4">
+        <v>52</v>
+      </c>
+      <c t="s" r="AL24" s="4">
+        <v>52</v>
+      </c>
+      <c r="AM24" s="2">
+        <v>1</v>
+      </c>
+      <c r="AN24" s="2">
+        <v>1</v>
+      </c>
+      <c t="s" r="AO24" s="4">
+        <v>53</v>
+      </c>
+      <c t="s" r="AP24" s="4">
+        <v>54</v>
+      </c>
+      <c t="s" r="AQ24" s="4">
+        <v>55</v>
+      </c>
+      <c t="s" r="AR24" s="4">
         <v>67</v>
       </c>
-      <c t="s" r="Q24" s="13">
-        <v>68</v>
-      </c>
-      <c t="s" r="R24" s="13">
-        <v>69</v>
-      </c>
-      <c t="s" r="S24" s="13">
-        <v>70</v>
-      </c>
-      <c t="s" r="T24" s="13">
-        <v>71</v>
-      </c>
-      <c t="s" r="U24" s="13">
-        <v>72</v>
-      </c>
-      <c t="s" r="V24" s="13">
-        <v>73</v>
-      </c>
-      <c t="s" r="W24" s="13">
-        <v>74</v>
-      </c>
-      <c t="s" r="X24" s="13">
-        <v>75</v>
-      </c>
-      <c t="s" r="Y24" s="13">
-        <v>76</v>
-      </c>
-      <c t="s" r="Z24" s="13">
-        <v>77</v>
-      </c>
-      <c t="s" r="AA24" s="13">
-        <v>78</v>
-      </c>
-      <c t="s" r="AB24" s="13">
-        <v>79</v>
-      </c>
-      <c t="s" r="AC24" s="13">
-        <v>80</v>
-      </c>
-      <c t="s" r="AD24" s="13">
-        <v>81</v>
-      </c>
-      <c t="s" r="AE24" s="13">
-        <v>82</v>
-      </c>
-      <c r="AF24" s="13"/>
-      <c t="s" r="AG24" s="13">
-        <v>83</v>
-      </c>
-      <c t="s" r="AH24" s="13">
-        <v>84</v>
-      </c>
-      <c t="s" r="AI24" s="13">
-        <v>85</v>
-      </c>
-      <c r="AJ24" s="14"/>
-      <c t="s" r="AK24" s="14">
-        <v>52</v>
-      </c>
-      <c t="s" r="AL24" s="14">
-        <v>52</v>
-      </c>
-      <c t="s" r="AM24" s="13">
-        <v>86</v>
-      </c>
-      <c t="s" r="AN24" s="13">
-        <v>86</v>
-      </c>
-      <c r="AO24" s="14"/>
-      <c r="AP24" s="14"/>
-      <c r="AQ24" s="14"/>
-      <c r="AR24" s="14"/>
-      <c r="AS24" s="14"/>
+      <c t="s" r="AS24" s="4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" ht="13.5" customHeight="1">
+      <c r="A25" s="2">
+        <v>19914</v>
+      </c>
+      <c r="B25" s="3">
+        <v>0</v>
+      </c>
+      <c t="s" r="C25" s="4">
+        <v>44</v>
+      </c>
+      <c t="s" r="D25" s="4">
+        <v>89</v>
+      </c>
+      <c t="s" r="E25" s="4">
+        <v>90</v>
+      </c>
+      <c t="s" r="F25" s="4">
+        <v>47</v>
+      </c>
+      <c t="s" r="G25" s="4">
+        <v>48</v>
+      </c>
+      <c t="s" r="H25" s="4">
+        <v>49</v>
+      </c>
+      <c t="s" r="I25" s="4">
+        <v>50</v>
+      </c>
+      <c t="s" r="J25" s="4">
+        <v>47</v>
+      </c>
+      <c t="s" r="K25" s="4">
+        <v>51</v>
+      </c>
+      <c t="s" r="L25" s="4">
+        <v>51</v>
+      </c>
+      <c r="M25" s="4"/>
+      <c t="s" r="N25" s="4">
+        <v>52</v>
+      </c>
+      <c r="O25" s="5">
+        <v>28714.359999999997</v>
+      </c>
+      <c r="P25" s="5">
+        <v>28714.359999999997</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>-0.0087965869946659003</v>
+      </c>
+      <c r="R25" s="7">
+        <v>325</v>
+      </c>
+      <c r="S25" s="6">
+        <v>-0.035608308605341255</v>
+      </c>
+      <c r="T25" s="6">
+        <v>0.27291786409308788</v>
+      </c>
+      <c r="U25" s="6">
+        <v>-0.0070100186805486867</v>
+      </c>
+      <c r="V25" s="6">
+        <v>0.028498180004708447</v>
+      </c>
+      <c r="W25" s="6">
+        <v>0.014167023050487631</v>
+      </c>
+      <c r="X25" s="8">
+        <v>30.855609134615385</v>
+      </c>
+      <c r="Y25" s="6">
+        <v>0.40384615384615385</v>
+      </c>
+      <c r="Z25" s="6">
+        <v>0.19711538461538461</v>
+      </c>
+      <c r="AA25" s="8">
+        <v>7.4241133738601821</v>
+      </c>
+      <c r="AB25" s="8">
+        <v>8.5097291891891889</v>
+      </c>
+      <c r="AC25" s="8">
+        <v>14.799942</v>
+      </c>
+      <c r="AD25" s="8">
+        <v>22.687980769230769</v>
+      </c>
+      <c r="AE25" s="6">
+        <v>0.51442307692307687</v>
+      </c>
+      <c r="AF25" s="9"/>
+      <c r="AG25" s="5">
+        <v>-713.87</v>
+      </c>
+      <c r="AH25" s="10">
+        <v>2</v>
+      </c>
+      <c r="AI25" s="11"/>
+      <c r="AJ25" s="12">
+        <v>45996</v>
+      </c>
+      <c t="s" r="AK25" s="4">
+        <v>52</v>
+      </c>
+      <c t="s" r="AL25" s="4">
+        <v>52</v>
+      </c>
+      <c r="AM25" s="2">
+        <v>1</v>
+      </c>
+      <c r="AN25" s="2">
+        <v>1</v>
+      </c>
+      <c t="s" r="AO25" s="4">
+        <v>53</v>
+      </c>
+      <c t="s" r="AP25" s="4">
+        <v>54</v>
+      </c>
+      <c t="s" r="AQ25" s="4">
+        <v>55</v>
+      </c>
+      <c t="s" r="AR25" s="4">
+        <v>91</v>
+      </c>
+      <c t="s" r="AS25" s="4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" ht="13.5" customHeight="1">
+      <c r="A26" s="2">
+        <v>19958</v>
+      </c>
+      <c r="B26" s="3">
+        <v>0</v>
+      </c>
+      <c t="s" r="C26" s="4">
+        <v>44</v>
+      </c>
+      <c t="s" r="D26" s="4">
+        <v>92</v>
+      </c>
+      <c t="s" r="E26" s="4">
+        <v>93</v>
+      </c>
+      <c t="s" r="F26" s="4">
+        <v>47</v>
+      </c>
+      <c t="s" r="G26" s="4">
+        <v>48</v>
+      </c>
+      <c t="s" r="H26" s="4">
+        <v>49</v>
+      </c>
+      <c t="s" r="I26" s="4">
+        <v>50</v>
+      </c>
+      <c t="s" r="J26" s="4">
+        <v>47</v>
+      </c>
+      <c t="s" r="K26" s="4">
+        <v>51</v>
+      </c>
+      <c t="s" r="L26" s="4">
+        <v>51</v>
+      </c>
+      <c r="M26" s="4"/>
+      <c t="s" r="N26" s="4">
+        <v>52</v>
+      </c>
+      <c r="O26" s="5">
+        <v>18040.459999999999</v>
+      </c>
+      <c r="P26" s="5">
+        <v>18040.459999999999</v>
+      </c>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="7">
+        <v>205</v>
+      </c>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6">
+        <v>0.40189848263292621</v>
+      </c>
+      <c r="U26" s="6">
+        <v>0.071394714990637723</v>
+      </c>
+      <c r="V26" s="6">
+        <v>0.032002149612593025</v>
+      </c>
+      <c r="W26" s="6">
+        <v>0.0029269486476508916</v>
+      </c>
+      <c r="X26" s="8">
+        <v>28.615227160493827</v>
+      </c>
+      <c r="Y26" s="6">
+        <v>0.46913580246913578</v>
+      </c>
+      <c r="Z26" s="6">
+        <v>0.07407407407407407</v>
+      </c>
+      <c r="AA26" s="8">
+        <v>7.7159015306122454</v>
+      </c>
+      <c r="AB26" s="8">
+        <v>5.7262487499999999</v>
+      </c>
+      <c r="AC26" s="8">
+        <v>13.125953000000001</v>
+      </c>
+      <c r="AD26" s="8">
+        <v>20.184979012345678</v>
+      </c>
+      <c r="AE26" s="6">
+        <v>0.62962962962962965</v>
+      </c>
+      <c r="AF26" s="9"/>
+      <c r="AG26" s="5">
+        <v>-1061.98</v>
+      </c>
+      <c r="AH26" s="10">
+        <v>3</v>
+      </c>
+      <c r="AI26" s="11"/>
+      <c r="AJ26" s="12">
+        <v>45937</v>
+      </c>
+      <c t="s" r="AK26" s="4">
+        <v>52</v>
+      </c>
+      <c t="s" r="AL26" s="4">
+        <v>52</v>
+      </c>
+      <c r="AM26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AN26" s="2">
+        <v>1</v>
+      </c>
+      <c t="s" r="AO26" s="4">
+        <v>53</v>
+      </c>
+      <c t="s" r="AP26" s="4">
+        <v>54</v>
+      </c>
+      <c t="s" r="AQ26" s="4">
+        <v>55</v>
+      </c>
+      <c t="s" r="AR26" s="4">
+        <v>94</v>
+      </c>
+      <c t="s" r="AS26" s="4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" ht="24.75" customHeight="1">
+      <c t="s" r="A27" s="13">
+        <v>95</v>
+      </c>
+      <c t="s" r="B27" s="13">
+        <v>96</v>
+      </c>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="14"/>
+      <c t="s" r="N27" s="14">
+        <v>52</v>
+      </c>
+      <c t="s" r="O27" s="13">
+        <v>97</v>
+      </c>
+      <c t="s" r="P27" s="13">
+        <v>98</v>
+      </c>
+      <c t="s" r="Q27" s="13">
+        <v>99</v>
+      </c>
+      <c t="s" r="R27" s="13">
+        <v>100</v>
+      </c>
+      <c t="s" r="S27" s="13">
+        <v>101</v>
+      </c>
+      <c t="s" r="T27" s="13">
+        <v>102</v>
+      </c>
+      <c t="s" r="U27" s="13">
+        <v>103</v>
+      </c>
+      <c t="s" r="V27" s="13">
+        <v>104</v>
+      </c>
+      <c t="s" r="W27" s="13">
+        <v>105</v>
+      </c>
+      <c t="s" r="X27" s="13">
+        <v>106</v>
+      </c>
+      <c t="s" r="Y27" s="13">
+        <v>107</v>
+      </c>
+      <c t="s" r="Z27" s="13">
+        <v>108</v>
+      </c>
+      <c t="s" r="AA27" s="13">
+        <v>109</v>
+      </c>
+      <c t="s" r="AB27" s="13">
+        <v>110</v>
+      </c>
+      <c t="s" r="AC27" s="13">
+        <v>111</v>
+      </c>
+      <c t="s" r="AD27" s="13">
+        <v>112</v>
+      </c>
+      <c t="s" r="AE27" s="13">
+        <v>113</v>
+      </c>
+      <c r="AF27" s="13"/>
+      <c t="s" r="AG27" s="13">
+        <v>114</v>
+      </c>
+      <c t="s" r="AH27" s="13">
+        <v>115</v>
+      </c>
+      <c t="s" r="AI27" s="13">
+        <v>116</v>
+      </c>
+      <c r="AJ27" s="14"/>
+      <c t="s" r="AK27" s="14">
+        <v>52</v>
+      </c>
+      <c t="s" r="AL27" s="14">
+        <v>52</v>
+      </c>
+      <c t="s" r="AM27" s="13">
+        <v>117</v>
+      </c>
+      <c t="s" r="AN27" s="13">
+        <v>117</v>
+      </c>
+      <c r="AO27" s="14"/>
+      <c r="AP27" s="14"/>
+      <c r="AQ27" s="14"/>
+      <c r="AR27" s="14"/>
+      <c r="AS27" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AS24" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:AS27" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>